<commit_message>
612 re-doing for IPv4
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBCFD7BA-9431-AB4E-AAD8-33062A368C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD411DD2-1DE1-E64D-BB05-828774E49A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="8" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="3" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="51">
   <si>
     <t>enable</t>
   </si>
@@ -54,9 +54,6 @@
     <t>hostname MS4</t>
   </si>
   <si>
-    <t>sdm prefer dual-ipv4-and-ipv6 default</t>
-  </si>
-  <si>
     <t>no ip domain-lookup</t>
   </si>
   <si>
@@ -84,19 +81,121 @@
     <t>hostname MS0</t>
   </si>
   <si>
-    <t>ipv6 unicast-routing</t>
-  </si>
-  <si>
     <t>hostname MS1</t>
   </si>
   <si>
+    <t>vlan 10</t>
+  </si>
+  <si>
+    <t>name LAB1</t>
+  </si>
+  <si>
+    <t>vlan 20</t>
+  </si>
+  <si>
+    <t>name LAB2</t>
+  </si>
+  <si>
+    <t>vlan 30</t>
+  </si>
+  <si>
+    <t>name ADMIN</t>
+  </si>
+  <si>
+    <t>vlan 40</t>
+  </si>
+  <si>
+    <t>name ACADEMIC</t>
+  </si>
+  <si>
+    <t>vlan 50</t>
+  </si>
+  <si>
+    <t>name SERVER</t>
+  </si>
+  <si>
+    <t>exit</t>
+  </si>
+  <si>
+    <t>interface vlan 10</t>
+  </si>
+  <si>
+    <t>no shutdown</t>
+  </si>
+  <si>
+    <t>interface vlan 20</t>
+  </si>
+  <si>
+    <t>interface vlan 30</t>
+  </si>
+  <si>
+    <t>interface vlan 40</t>
+  </si>
+  <si>
+    <t>interface vlan 50</t>
+  </si>
+  <si>
+    <t>interface gi1/0/1</t>
+  </si>
+  <si>
+    <t>switchport mode trunk</t>
+  </si>
+  <si>
+    <t>interface gi1/0/2</t>
+  </si>
+  <si>
+    <t>interface gi1/0/4</t>
+  </si>
+  <si>
+    <t>interface gi1/0/3</t>
+  </si>
+  <si>
+    <t>interface gi0/1</t>
+  </si>
+  <si>
     <t>erase startup-config</t>
   </si>
   <si>
+    <t>switchport trunk encapsulation dot1q</t>
+  </si>
+  <si>
     <t>hostname Firewall22</t>
   </si>
   <si>
+    <t>switchport mode access</t>
+  </si>
+  <si>
+    <t>switchport access vlan 50</t>
+  </si>
+  <si>
     <t>write erase</t>
+  </si>
+  <si>
+    <t>ip routing</t>
+  </si>
+  <si>
+    <t>ip address 192.168.10.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 192.168.20.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 192.168.30.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 192.168.40.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 192.168.50.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>access-list 100 permit ip 192.168.50.0 0.0.0.255 any</t>
+  </si>
+  <si>
+    <t>access-list 100 deny ip any any</t>
+  </si>
+  <si>
+    <t>ip access-group 100 in</t>
   </si>
 </sst>
 </file>
@@ -495,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34311B4-1E30-6D40-A73D-B4C7308E242A}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.83203125" customWidth="1"/>
@@ -518,22 +617,62 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -543,7 +682,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
@@ -561,27 +700,67 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -591,7 +770,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC59594-6BB4-1E4A-B489-1D5AC66DAC96}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
@@ -609,27 +788,67 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -639,7 +858,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
@@ -657,37 +876,67 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>13</v>
+      <c r="A6" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
-        <v>7</v>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -697,7 +946,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48880218-5589-A547-BB90-D873A156AAD1}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.5" customWidth="1"/>
@@ -715,27 +964,67 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -745,7 +1034,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFEE1F6-6AF7-454F-BBB3-C95B039FA8B6}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -763,27 +1052,107 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -793,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -811,32 +1180,319 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>13</v>
+      <c r="A4" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="3"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="3"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="3"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" s="3"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="3"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="3"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="3"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" s="3"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="3"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="3"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="3"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="3"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -864,22 +1520,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -897,17 +1553,17 @@
   <sheetData>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
612 working excep MS2
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD411DD2-1DE1-E64D-BB05-828774E49A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D88899A-C3C8-DB43-91FC-8D5791F84553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="3" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="55">
   <si>
     <t>enable</t>
   </si>
@@ -57,15 +57,9 @@
     <t>no ip domain-lookup</t>
   </si>
   <si>
-    <t>Exit</t>
-  </si>
-  <si>
     <t>write memory</t>
   </si>
   <si>
-    <t>Reload</t>
-  </si>
-  <si>
     <t>hostname MS3</t>
   </si>
   <si>
@@ -156,6 +150,9 @@
     <t>erase startup-config</t>
   </si>
   <si>
+    <t>interface range fa0/1-24</t>
+  </si>
+  <si>
     <t>switchport trunk encapsulation dot1q</t>
   </si>
   <si>
@@ -189,13 +186,28 @@
     <t>ip address 192.168.50.1 255.255.255.0</t>
   </si>
   <si>
-    <t>access-list 100 permit ip 192.168.50.0 0.0.0.255 any</t>
-  </si>
-  <si>
-    <t>access-list 100 deny ip any any</t>
-  </si>
-  <si>
-    <t>ip access-group 100 in</t>
+    <t>no shut</t>
+  </si>
+  <si>
+    <t>switchport access vlan 10</t>
+  </si>
+  <si>
+    <t>switchport access vlan 20</t>
+  </si>
+  <si>
+    <t>switchport access vlan 30</t>
+  </si>
+  <si>
+    <t>switchport access vlan 40</t>
+  </si>
+  <si>
+    <t>interface gi1/1</t>
+  </si>
+  <si>
+    <t>interface gi1/2</t>
+  </si>
+  <si>
+    <t>spanning-tree vlan 10,20,30,40,50 priority 4096</t>
   </si>
 </sst>
 </file>
@@ -594,7 +606,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34311B4-1E30-6D40-A73D-B4C7308E242A}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.83203125" customWidth="1"/>
@@ -620,60 +632,64 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>23</v>
-      </c>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -682,7 +698,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
@@ -700,7 +716,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -708,59 +724,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -788,7 +799,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -796,59 +807,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +882,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -884,59 +890,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -946,7 +947,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48880218-5589-A547-BB90-D873A156AAD1}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.5" customWidth="1"/>
@@ -964,7 +965,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -972,59 +973,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>31</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1034,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFEE1F6-6AF7-454F-BBB3-C95B039FA8B6}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1052,7 +1048,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
@@ -1060,99 +1056,74 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
+      <c r="A6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>16</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>32</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1162,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A83"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -1180,110 +1151,128 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>6</v>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>0</v>
+      <c r="A12" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A18" s="3"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
+      <c r="A21" s="3" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="3"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
+      <c r="A24" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3"/>
+      <c r="A26" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>43</v>
-      </c>
+      <c r="A27" s="3"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3"/>
+      <c r="A28" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="3"/>
+      <c r="A30" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="3"/>
@@ -1294,11 +1283,13 @@
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3"/>
+      <c r="A33" s="3" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
@@ -1306,45 +1297,51 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
+      <c r="A37" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="3"/>
+      <c r="A38" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="A39" s="3"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" s="3"/>
+      <c r="A40" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
-        <v>45</v>
-      </c>
+      <c r="A41" s="3"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" s="3"/>
+      <c r="A42" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" s="3"/>
+      <c r="A45" s="3" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
@@ -1352,34 +1349,38 @@
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" s="3"/>
+      <c r="A49" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
-        <v>25</v>
-      </c>
+      <c r="A50" s="3"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" s="3"/>
+      <c r="A51" s="3" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" s="3"/>
+      <c r="A52" s="3" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="A53" s="3"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" s="3"/>
+      <c r="A54" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
@@ -1387,7 +1388,7 @@
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
@@ -1395,105 +1396,23 @@
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="3"/>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
-        <v>30</v>
-      </c>
+      <c r="A61" s="3"/>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="A62" s="3"/>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="3"/>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="3"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A69" s="3"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>50</v>
-      </c>
+      <c r="A64" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1502,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -1520,22 +1439,50 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="3"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1553,17 +1500,17 @@
   <sheetData>
     <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
612 MS2-MS1 not working
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D88899A-C3C8-DB43-91FC-8D5791F84553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB214A52-291C-2048-9782-677B9C34CE14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="75">
   <si>
     <t>enable</t>
   </si>
@@ -186,6 +186,9 @@
     <t>ip address 192.168.50.1 255.255.255.0</t>
   </si>
   <si>
+    <t>conf t</t>
+  </si>
+  <si>
     <t>no shut</t>
   </si>
   <si>
@@ -208,6 +211,63 @@
   </si>
   <si>
     <t>spanning-tree vlan 10,20,30,40,50 priority 4096</t>
+  </si>
+  <si>
+    <t>! Crear VLAN 50</t>
+  </si>
+  <si>
+    <t>! Configurar puertos de PCs en VLAN 50</t>
+  </si>
+  <si>
+    <t>! Puerto hacia firewall como access también</t>
+  </si>
+  <si>
+    <t>! Interfaz hacia MS2 (VLAN 50)</t>
+  </si>
+  <si>
+    <t>ip address 192.168.50.254 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t>switchport access vlan 99</t>
+  </si>
+  <si>
+    <t>vlan 99</t>
+  </si>
+  <si>
+    <t>name BACKBONE</t>
+  </si>
+  <si>
+    <t>interface vlan 99</t>
+  </si>
+  <si>
+    <t>ip address 192.168.99.2 255.255.255.0</t>
+  </si>
+  <si>
+    <t>ip route 192.168.50.0 255.255.255.0 192.168.99.1</t>
+  </si>
+  <si>
+    <t>! Habilitar routing</t>
+  </si>
+  <si>
+    <t>description To_MS2_VLAN50</t>
+  </si>
+  <si>
+    <t>! Interfaz hacia MS1 (backbone VLAN 99)</t>
+  </si>
+  <si>
+    <t>description To_MS1_Backbone</t>
+  </si>
+  <si>
+    <t>! Rutas (opcional si MS1 tiene estática)</t>
+  </si>
+  <si>
+    <t>! ip route 192.168.99.0 255.255.255.0 gi1/2</t>
+  </si>
+  <si>
+    <t>! ip route 192.168.50.0 255.255.255.0 gi1/1</t>
   </si>
 </sst>
 </file>
@@ -229,12 +289,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -286,12 +352,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,7 +731,7 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
@@ -756,7 +823,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
@@ -839,7 +906,7 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
@@ -864,7 +931,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
@@ -939,6 +1006,109 @@
       <c r="A18" t="s">
         <v>4</v>
       </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="5"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="5"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="5"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="5"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="5"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1005,7 +1175,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -1133,7 +1303,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -1235,7 +1405,7 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
@@ -1253,7 +1423,7 @@
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
@@ -1271,7 +1441,7 @@
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
@@ -1289,7 +1459,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
@@ -1307,7 +1477,7 @@
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
@@ -1396,7 +1566,7 @@
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
@@ -1413,6 +1583,103 @@
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="4"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" s="5"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" s="5"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A85" s="5"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A86" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A87" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A88" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A89" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A90" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A91" s="5"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A92" s="5"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A93" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A94" s="5"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A95" s="5"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A96" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A97" s="5"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A98" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A99" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A100" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1421,7 +1688,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -1447,7 +1714,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -1462,7 +1729,7 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
@@ -1482,6 +1749,113 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="5"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="5"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="5"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
612 red-working, additional permit ping any rules Firewall22
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER-IPv4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB214A52-291C-2048-9782-677B9C34CE14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA4C8C4-9B4A-884F-96F9-423CDEA1300F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="2" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="96">
   <si>
     <t>enable</t>
   </si>
@@ -186,9 +186,6 @@
     <t>ip address 192.168.50.1 255.255.255.0</t>
   </si>
   <si>
-    <t>conf t</t>
-  </si>
-  <si>
     <t>no shut</t>
   </si>
   <si>
@@ -204,77 +201,143 @@
     <t>switchport access vlan 40</t>
   </si>
   <si>
-    <t>interface gi1/1</t>
-  </si>
-  <si>
-    <t>interface gi1/2</t>
-  </si>
-  <si>
-    <t>spanning-tree vlan 10,20,30,40,50 priority 4096</t>
-  </si>
-  <si>
-    <t>! Crear VLAN 50</t>
-  </si>
-  <si>
-    <t>! Configurar puertos de PCs en VLAN 50</t>
-  </si>
-  <si>
-    <t>! Puerto hacia firewall como access también</t>
-  </si>
-  <si>
-    <t>! Interfaz hacia MS2 (VLAN 50)</t>
-  </si>
-  <si>
-    <t>ip address 192.168.50.254 255.255.255.0</t>
-  </si>
-  <si>
-    <t>ip address 192.168.99.1 255.255.255.0</t>
-  </si>
-  <si>
-    <t>switchport access vlan 99</t>
-  </si>
-  <si>
-    <t>vlan 99</t>
-  </si>
-  <si>
-    <t>name BACKBONE</t>
-  </si>
-  <si>
-    <t>interface vlan 99</t>
-  </si>
-  <si>
-    <t>ip address 192.168.99.2 255.255.255.0</t>
-  </si>
-  <si>
-    <t>ip route 192.168.50.0 255.255.255.0 192.168.99.1</t>
-  </si>
-  <si>
-    <t>! Habilitar routing</t>
-  </si>
-  <si>
-    <t>description To_MS2_VLAN50</t>
-  </si>
-  <si>
-    <t>! Interfaz hacia MS1 (backbone VLAN 99)</t>
-  </si>
-  <si>
-    <t>description To_MS1_Backbone</t>
-  </si>
-  <si>
-    <t>! Rutas (opcional si MS1 tiene estática)</t>
-  </si>
-  <si>
-    <t>! ip route 192.168.99.0 255.255.255.0 gi1/2</t>
-  </si>
-  <si>
-    <t>! ip route 192.168.50.0 255.255.255.0 gi1/1</t>
+    <t>no switchport</t>
+  </si>
+  <si>
+    <t>ip address 10.0.0.1 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip route 192.168.50.0 255.255.255.0 10.0.0.2</t>
+  </si>
+  <si>
+    <t>spanning-tree vlan 10,20,30,40 priority 4096</t>
+  </si>
+  <si>
+    <t>interface GigabitEthernet1/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> nameif inside</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> security-level 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ip address 10.0.0.2 255.255.255.252</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no shutdown</t>
+  </si>
+  <si>
+    <t>interface GigabitEthernet1/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> nameif dmz</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> security-level 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ip address 10.0.0.5 255.255.255.252</t>
+  </si>
+  <si>
+    <t>route inside 192.168.0.0 255.255.0.0 10.0.0.1</t>
+  </si>
+  <si>
+    <t>route dmz 192.168.50.0 255.255.255.0 10.0.0.6</t>
+  </si>
+  <si>
+    <t>access-list INSIDE_IN extended permit ip 192.168.0.0 255.255.0.0 192.168.50.0 255.255.255.0</t>
+  </si>
+  <si>
+    <t>access-group INSIDE_IN in interface inside</t>
+  </si>
+  <si>
+    <t>Enlace</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>MS1 &lt;-&gt; Firewall2</t>
+  </si>
+  <si>
+    <t>10.0.0.0/30</t>
+  </si>
+  <si>
+    <t>MS1 (Gi1/0/3): 10.0.0.1</t>
+  </si>
+  <si>
+    <t>Firewall2 &lt;-&gt; MS2</t>
+  </si>
+  <si>
+    <t>10.0.0.4/30</t>
+  </si>
+  <si>
+    <t>MS2 (Gi0/1): 10.0.0.6</t>
+  </si>
+  <si>
+    <t>192.168.50.0/24</t>
+  </si>
+  <si>
+    <t>Gateway (MS2): 192.168.50.1</t>
+  </si>
+  <si>
+    <t>Firewall2 (Gi1/1): 10.0.0.2</t>
+  </si>
+  <si>
+    <t>Firewall2 (Gi1/2): 10.0.0.5</t>
+  </si>
+  <si>
+    <t>XXXXXXX</t>
+  </si>
+  <si>
+    <t>VLAN 50 (SERVERS)</t>
+  </si>
+  <si>
+    <t>Origen</t>
+  </si>
+  <si>
+    <t>Destino</t>
+  </si>
+  <si>
+    <t>ip address 10.0.0.6 255.255.255.252</t>
+  </si>
+  <si>
+    <t>ip route 0.0.0.0 0.0.0.0 10.0.0.5</t>
+  </si>
+  <si>
+    <t>policy-map global_policy</t>
+  </si>
+  <si>
+    <t>class inspection_default</t>
+  </si>
+  <si>
+    <t>inspect icmp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface range fa0/1-24 </t>
+  </si>
+  <si>
+    <t>access-list ICMP_ALLOW extended permit icmp any any echo</t>
+  </si>
+  <si>
+    <t>access-list ICMP_ALLOW extended permit icmp any any echo-reply</t>
+  </si>
+  <si>
+    <t>access-list ICMP_ALLOW extended permit icmp any any unreachable</t>
+  </si>
+  <si>
+    <t>access-group ICMP_ALLOW in interface inside</t>
+  </si>
+  <si>
+    <t>access-group ICMP_ALLOW in interface dmz</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -288,22 +351,29 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -348,17 +418,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -731,7 +858,7 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
@@ -823,7 +950,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
@@ -906,7 +1033,7 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
@@ -931,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
@@ -957,158 +1084,138 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="4"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="5"/>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="5"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" s="5"/>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" s="5"/>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" s="5"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1175,7 +1282,7 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
@@ -1303,7 +1410,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A100"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -1330,9 +1437,12 @@
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>41</v>
       </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="3"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
@@ -1378,14 +1488,10 @@
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="A16" s="3"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A17" s="3"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
@@ -1405,7 +1511,7 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
@@ -1423,7 +1529,7 @@
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
@@ -1441,7 +1547,7 @@
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
@@ -1459,26 +1565,20 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="3"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="A36" s="3"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
-        <v>46</v>
-      </c>
+      <c r="A37" s="3"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
-        <v>48</v>
-      </c>
+      <c r="A38" s="3"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" s="3"/>
@@ -1531,14 +1631,10 @@
       <c r="A50" s="3"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
-        <v>32</v>
-      </c>
+      <c r="A51" s="3"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
-        <v>29</v>
-      </c>
+      <c r="A52" s="3"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="3"/>
@@ -1557,129 +1653,76 @@
       <c r="A56" s="3"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" s="3"/>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="3"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="3"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" s="3"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" s="3"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" s="3"/>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A63" s="3"/>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A64" s="4"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A78" s="5"/>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A79" s="5"/>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A80" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A81" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A82" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A83" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A84" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A85" s="5"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A86" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A87" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A88" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A89" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A90" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A91" s="5"/>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A92" s="5"/>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A93" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A94" s="5"/>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A95" s="5"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A96" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A97" s="5"/>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A98" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A99" s="5" t="s">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="3"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="3"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A100" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1688,175 +1731,255 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
+    <col min="1" max="1" width="89.6640625" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B3" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B4" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="5"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="5"/>
+      <c r="A31" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="5" t="s">
-        <v>59</v>
+      <c r="A32" s="3" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
-        <v>53</v>
+      <c r="A33" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="5" t="s">
-        <v>69</v>
+      <c r="A34" s="3" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
-        <v>60</v>
+      <c r="A35" s="3" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="A36" s="3"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="5"/>
+      <c r="A37" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
-        <v>61</v>
+      <c r="A38" s="3"/>
+    </row>
+    <row r="39" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
-        <v>23</v>
+      <c r="A42" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" s="5"/>
+      <c r="A43" s="3" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="s">
-        <v>72</v>
+      <c r="A44" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" s="5" t="s">
-        <v>73</v>
-      </c>
+      <c r="A45" s="3"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>74</v>
+      <c r="A46" s="3"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>4</v>
+      <c r="A48" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>